<commit_message>
fix: Set age default to 18 in loan form (BUG-002)
- Add age: 18 to formData initialization in useLoanForm.ts
- Fix age field defaulting to undefined instead of 18
- Create comprehensive test suite (8 tests) for age field in useLoanForm.test.ts
- Age now correctly defaults as number type, persists through form navigation
- Validation properly accepts age 18+ as valid
</commit_message>
<xml_diff>
--- a/BUG_TRACKER.xlsx
+++ b/BUG_TRACKER.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ashh\Downloads\CreditGenAI_current\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CE63C778-1C01-40AB-9B90-0DA38B4896C6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{82F5D3A7-3944-458B-9165-CE1E0D1C9AC5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="19">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="25">
   <si>
     <t>Bug_ID</t>
   </si>
@@ -77,6 +77,24 @@
   </si>
   <si>
     <t>BUG-002</t>
+  </si>
+  <si>
+    <t>Age field defaults to Undefined in Loan Form</t>
+  </si>
+  <si>
+    <t>Age field in Personal Details step doesn't default to 18. Displays 18 visually but stores undefined internally</t>
+  </si>
+  <si>
+    <t>useLoanForm.ts missing age in formData initialization</t>
+  </si>
+  <si>
+    <t>Add age: 18 to formData state initialization</t>
+  </si>
+  <si>
+    <t>src/hooks/useLoanForm.ts</t>
+  </si>
+  <si>
+    <t>Yes - userLoanForm.test.ts</t>
   </si>
 </sst>
 </file>
@@ -368,6 +386,9 @@
       </border>
     </dxf>
     <dxf>
+      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
       <font>
         <b/>
         <i val="0"/>
@@ -386,9 +407,6 @@
       </font>
       <alignment horizontal="left" vertical="top" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
-    <dxf>
-      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleMedium4"/>
   <extLst>
@@ -403,7 +421,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{AC22DD88-E891-445F-AA67-574A20E00B46}" name="Table4" displayName="Table4" ref="A1:I1048576" totalsRowShown="0" headerRowDxfId="9" dataDxfId="10">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{AC22DD88-E891-445F-AA67-574A20E00B46}" name="Table4" displayName="Table4" ref="A1:I1048576" totalsRowShown="0" headerRowDxfId="10" dataDxfId="9">
   <autoFilter ref="A1:I1048576" xr:uid="{AC22DD88-E891-445F-AA67-574A20E00B46}"/>
   <tableColumns count="9">
     <tableColumn id="1" xr3:uid="{0A361A17-691A-4EB7-80A3-B9DB31762CD0}" name="Bug_ID" dataDxfId="8"/>
@@ -813,12 +831,33 @@
         <v>16</v>
       </c>
     </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:9" ht="46.8" x14ac:dyDescent="0.3">
       <c r="A3" s="5" t="s">
         <v>18</v>
       </c>
       <c r="B3" s="6">
         <v>46126</v>
+      </c>
+      <c r="C3" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="D3" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="E3" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="F3" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="G3" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="H3" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="I3" s="5" t="s">
+        <v>24</v>
       </c>
     </row>
   </sheetData>

</xml_diff>